<commit_message>
Added Taxonomy of QAs and Tactics to Model
</commit_message>
<xml_diff>
--- a/semantic model development/foundational_semantic_model_generator/src/foundational_semantic_model_generator/input/SMS + Multicase/quality-attribute-classification-overview.xlsx
+++ b/semantic model development/foundational_semantic_model_generator/src/foundational_semantic_model_generator/input/SMS + Multicase/quality-attribute-classification-overview.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phili\Dropbox\01_Dev\02_QualiTact\Repository\QualiTact\semantic model development\fundational_semantic_model_generator\src\foundational_semantic_model_generator\input\SMS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phili\Dropbox\01_Dev\02_QualiTact\Repository\QualiTact\semantic model development\foundational_semantic_model_generator\src\foundational_semantic_model_generator\input\SMS + Multicase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B22C53-31FA-4770-AF28-440CB878F227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEE8F2E0-77DB-424D-9055-3C232D56D9FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13416" yWindow="4992" windowWidth="16416" windowHeight="5832" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sheet1!$F$1:$F$57</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tabelle1!$A$1:$F$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tabelle1!$A$1:$F$58</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,14 +39,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="139">
   <si>
     <t>Quality Attribute</t>
   </si>
   <si>
-    <t>Sub-Charateristic</t>
-  </si>
-  <si>
     <t>Functional completeness</t>
   </si>
   <si>
@@ -438,6 +435,27 @@
   </si>
   <si>
     <t>https://doi.org/10.1109/JPROC.2009.2036747</t>
+  </si>
+  <si>
+    <t>Characteristic</t>
+  </si>
+  <si>
+    <t>SubCharacteristic</t>
+  </si>
+  <si>
+    <t>Integrity</t>
+  </si>
+  <si>
+    <t>Modifiability</t>
+  </si>
+  <si>
+    <t>Testability</t>
+  </si>
+  <si>
+    <t>Verifiability</t>
+  </si>
+  <si>
+    <t>Includes all quality attributes, that are not included within a characteristic by ISO25059</t>
   </si>
 </sst>
 </file>
@@ -808,7 +826,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="31.44140625" style="2" customWidth="1"/>
@@ -820,691 +838,700 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>48</v>
-      </c>
       <c r="E1" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>132</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E14" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="F14" s="6" t="s">
         <v>121</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G17" s="1"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G18" s="1"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G19" s="1"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G20" s="1"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>132</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G21" s="1"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E22" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="F22" s="6" t="s">
         <v>123</v>
-      </c>
-      <c r="F22" s="6" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G23" s="1"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>24</v>
+        <v>134</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G25" s="1"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E26" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F26" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="F26" s="6" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E29" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="F29" s="6" t="s">
         <v>129</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>132</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>32</v>
+        <v>135</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
@@ -1512,104 +1539,108 @@
         <v>98</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>105</v>
+        <v>56</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D36" s="3"/>
+      <c r="E36" s="4" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>102</v>
+        <v>49</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D37" s="3" t="s">
-        <v>57</v>
+        <v>132</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>132</v>
+        <v>92</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D38" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D38" s="3"/>
-      <c r="E38" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>105</v>
+      <c r="E38" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>21</v>
+        <v>55</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E39" s="5" t="s">
-        <v>75</v>
+        <v>132</v>
+      </c>
+      <c r="D39" s="3"/>
+      <c r="E39" s="4" t="s">
+        <v>113</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="G39" s="1"/>
+        <v>104</v>
+      </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D40" s="3"/>
-      <c r="E40" s="4" t="s">
-        <v>95</v>
+        <v>20</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>74</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>105</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="G40" s="1"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D41" s="3" t="s">
-        <v>56</v>
-      </c>
+        <v>132</v>
+      </c>
+      <c r="D41" s="3"/>
       <c r="E41" s="4" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
@@ -1617,135 +1648,140 @@
         <v>98</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>117</v>
+        <v>88</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>105</v>
+        <v>115</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>53</v>
+        <v>133</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>54</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="F45" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="G45" s="1"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>57</v>
+        <v>133</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>52</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>107</v>
+        <v>75</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>105</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="G46" s="1"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>98</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D48" s="3"/>
+        <v>43</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>56</v>
+      </c>
       <c r="E48" s="4" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -1753,59 +1789,57 @@
         <v>98</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>55</v>
-      </c>
+        <v>132</v>
+      </c>
+      <c r="D49" s="3"/>
       <c r="E49" s="4" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>6</v>
+        <v>136</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>42</v>
+        <v>5</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="F51" s="6" t="s">
-        <v>128</v>
+        <v>61</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
@@ -1813,50 +1847,53 @@
         <v>98</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>104</v>
+        <v>126</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>52</v>
+        <v>99</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>51</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>109</v>
+        <v>71</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>52</v>
+        <v>132</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>71</v>
+        <v>108</v>
       </c>
       <c r="F54" s="2" t="s">
         <v>104</v>
@@ -1864,77 +1901,97 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E55" s="4" t="s">
         <v>70</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>111</v>
+        <v>69</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="E57" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>98</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="F58" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="F57" s="6" t="s">
-        <v>126</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F57" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:F58" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="F42" r:id="rId1" xr:uid="{12524EF2-6C26-494C-AC48-F20172DBADD2}"/>
+    <hyperlink ref="F43" r:id="rId1" xr:uid="{12524EF2-6C26-494C-AC48-F20172DBADD2}"/>
     <hyperlink ref="F13" r:id="rId2" xr:uid="{1B9400A8-CB8C-460D-BE12-FD0068C7B786}"/>
     <hyperlink ref="F26" r:id="rId3" xr:uid="{6874A7DA-EC14-494B-9F71-C61827E58D0F}"/>
     <hyperlink ref="F14" r:id="rId4" xr:uid="{8A5F354D-9CD2-4978-8B8C-C054DB95431A}"/>
     <hyperlink ref="F22" r:id="rId5" xr:uid="{CB0F106C-41BE-41BA-B8D7-E0B4E40DC97B}"/>
-    <hyperlink ref="F57" r:id="rId6" xr:uid="{F7332246-A7D3-4F45-A189-317E7C235C0E}"/>
-    <hyperlink ref="F51" r:id="rId7" xr:uid="{2C183057-0DD2-4D18-9078-9368E8048C79}"/>
+    <hyperlink ref="F58" r:id="rId6" xr:uid="{F7332246-A7D3-4F45-A189-317E7C235C0E}"/>
+    <hyperlink ref="F52" r:id="rId7" xr:uid="{2C183057-0DD2-4D18-9078-9368E8048C79}"/>
     <hyperlink ref="F29" r:id="rId8" xr:uid="{FF79D626-7162-40FA-835A-DFF5481CC520}"/>
-    <hyperlink ref="F37" r:id="rId9" xr:uid="{49C558A6-63EF-4A0C-BC30-D5B057993419}"/>
+    <hyperlink ref="F38" r:id="rId9" xr:uid="{49C558A6-63EF-4A0C-BC30-D5B057993419}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1947,287 +2004,287 @@
   <sheetData>
     <row r="1" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F17" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F18" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F19" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F20" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F22" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="24" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F25" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F26" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F27" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="28" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="29" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F29" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="31" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F31" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F32" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F33" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="34" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F34" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="35" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F35" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="36" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F36" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="37" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F37" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="38" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F38" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="39" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F39" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F40" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="41" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F41" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="42" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F42" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="43" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F43" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F44" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="45" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F45" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="46" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F46" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="47" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F47" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="48" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F48" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="49" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F49" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="50" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F50" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F51" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="52" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F52" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="53" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F53" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="54" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F54" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="55" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F55" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="56" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F56" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="57" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F57" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>